<commit_message>
Update project files and remove frontend artifacts
</commit_message>
<xml_diff>
--- a/chemical_adsorbent_report.xlsx
+++ b/chemical_adsorbent_report.xlsx
@@ -9,16 +9,17 @@
   <sheets>
     <sheet name="Visualizations" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Dataset" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Training Data" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Testing &amp; Predictions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="All Predictions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Metal Combinations" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Model Metrics" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Coefficients" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Statistical Summary" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Correlation Matrix" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Graph Analysis" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="All Predictions Graphs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dataset" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Training Data" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Testing &amp; Predictions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="All Predictions" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Metal Combinations" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Model Metrics" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Coefficients" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Statistical Summary" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Correlation Matrix" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Graph Analysis" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -191,6 +192,89 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="15240000" cy="10668000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>61</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9144000" cy="7620000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>16</col>
+      <colOff>0</colOff>
+      <row>61</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="12192000" cy="6096000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -507,6 +591,198 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Coefficient</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Abs_Coefficient</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Metal_Mn</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>-10.98707973244456</v>
+      </c>
+      <c r="C2" t="n">
+        <v>10.98707973244456</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Metal_Pb</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>9.040480708412423</v>
+      </c>
+      <c r="C3" t="n">
+        <v>9.040480708412423</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Adsorbent_Biochar</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>-6.105736842622738</v>
+      </c>
+      <c r="C4" t="n">
+        <v>6.105736842622738</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Adsorbent_Chitosan composite</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>5.881827924216666</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5.881827924216666</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Temp (°C)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>-2.309184105167655</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2.309184105167655</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Metal_Cu</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1.946599024032162</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.946599024032162</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Time (min)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.6229174631890663</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.6229174631890663</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>pH</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.4844557363162729</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.4844557363162729</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Adsorbent_Activated Carbon</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.2239089184060762</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.2239089184060762</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RPM</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.09274999215494417</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.09274999215494417</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Dosage (g/L)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.01038195771982011</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.01038195771982011</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C0 (mg/L)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -846,7 +1122,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1174,7 +1450,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1491,6 +1767,20 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2978,7 +3268,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3974,7 +4264,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4400,7 +4690,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6002,7 +6292,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9728,7 +10018,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9814,196 +10104,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Coefficient</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Abs_Coefficient</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Metal_Mn</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>-10.98707973244456</v>
-      </c>
-      <c r="C2" t="n">
-        <v>10.98707973244456</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Metal_Pb</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>9.040480708412423</v>
-      </c>
-      <c r="C3" t="n">
-        <v>9.040480708412423</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Adsorbent_Biochar</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>-6.105736842622738</v>
-      </c>
-      <c r="C4" t="n">
-        <v>6.105736842622738</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Adsorbent_Chitosan composite</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>5.881827924216666</v>
-      </c>
-      <c r="C5" t="n">
-        <v>5.881827924216666</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Temp (°C)</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>-2.309184105167655</v>
-      </c>
-      <c r="C6" t="n">
-        <v>2.309184105167655</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Metal_Cu</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1.946599024032162</v>
-      </c>
-      <c r="C7" t="n">
-        <v>1.946599024032162</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Time (min)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0.6229174631890663</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.6229174631890663</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>pH</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0.4844557363162729</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.4844557363162729</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Adsorbent_Activated Carbon</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0.2239089184060762</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0.2239089184060762</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>RPM</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.09274999215494417</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0.09274999215494417</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Dosage (g/L)</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.01038195771982011</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0.01038195771982011</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>C0 (mg/L)</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>